<commit_message>
Fix current Higashihiroshima sake catalog gaps
</commit_message>
<xml_diff>
--- a/東広島市_安芸津・黒瀬エリア3蔵_主要日本酒一覧.xlsx
+++ b/東広島市_安芸津・黒瀬エリア3蔵_主要日本酒一覧.xlsx
@@ -209,7 +209,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_573163" displayName="T_573163" ref="A4:H10" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T_515919" displayName="T_515919" ref="A4:H10" headerRowCount="1">
   <autoFilter ref="A4:H10"/>
   <tableColumns count="8">
     <tableColumn id="1" name="エリア"/>
@@ -226,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T_839278" displayName="T_839278" ref="A4:R25" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T_845705" displayName="T_845705" ref="A4:R25" headerRowCount="1">
   <autoFilter ref="A4:R25"/>
   <tableColumns count="18">
     <tableColumn id="1" name="エリア"/>
@@ -253,7 +253,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T_565664" displayName="T_565664" ref="A4:M19" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T_726924" displayName="T_726924" ref="A4:M19" headerRowCount="1">
   <autoFilter ref="A4:M19"/>
   <tableColumns count="13">
     <tableColumn id="1" name="酒蔵"/>
@@ -275,7 +275,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T_930275" displayName="T_930275" ref="A4:B9" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T_560804" displayName="T_560804" ref="A4:B9" headerRowCount="1">
   <autoFilter ref="A4:B9"/>
   <tableColumns count="2">
     <tableColumn id="1" name="基準"/>
@@ -804,7 +804,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q5" s="7" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="P6" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q6" s="9" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="P8" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q8" s="9" t="inlineStr">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="P10" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q10" s="9" t="inlineStr">
@@ -1744,7 +1744,7 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="P12" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q12" s="9" t="inlineStr">
@@ -1920,7 +1920,7 @@
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="P14" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q14" s="9" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="P16" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q16" s="9" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="P18" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q18" s="9" t="inlineStr">
@@ -2421,7 +2421,7 @@
       <c r="L19" s="7" t="inlineStr"/>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>冷酒 / 常温 / 熱燗</t>
+          <t>冷酒 / 常温</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q19" s="7" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="R19" s="7" t="inlineStr">
         <is>
-          <t>https://www.tsukasyuzou.jp/products/於多福-純米-1800ml</t>
+          <t>https://www.tsukasyuzou.jp/products/火入れ-9代目於多福-純米大吟醸-720ml-1800ml</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       <c r="L20" s="9" t="inlineStr"/>
       <c r="M20" s="9" t="inlineStr">
         <is>
-          <t>冷酒 / 常温 / 熱燗</t>
+          <t>冷酒 / 常温 / ロック</t>
         </is>
       </c>
       <c r="N20" s="9" t="inlineStr">
@@ -2520,7 +2520,7 @@
       </c>
       <c r="P20" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q20" s="9" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="R20" s="9" t="inlineStr">
         <is>
-          <t>https://www.tsukasyuzou.jp/products/於多福-純米-1800ml</t>
+          <t>https://www.tsukasyuzou.jp/products/9代目於多福-すずかぜ-720ml</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q21" s="7" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="P22" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q22" s="9" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q23" s="7" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="P24" s="9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q24" s="9" t="inlineStr">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="Q25" s="7" t="inlineStr">
@@ -3724,7 +3724,7 @@
       <c r="G15" s="7" t="inlineStr"/>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>冷酒 / 常温 / 熱燗</t>
+          <t>冷酒 / 常温</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
@@ -3749,7 +3749,7 @@
       </c>
       <c r="M15" s="8" t="inlineStr">
         <is>
-          <t>https://www.tsukasyuzou.jp/products/於多福-純米-1800ml</t>
+          <t>https://www.tsukasyuzou.jp/products/火入れ-9代目於多福-純米大吟醸-720ml-1800ml</t>
         </is>
       </c>
     </row>
@@ -3783,7 +3783,7 @@
       <c r="G16" s="9" t="inlineStr"/>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>冷酒 / 常温 / 熱燗</t>
+          <t>冷酒 / 常温 / ロック</t>
         </is>
       </c>
       <c r="I16" s="9" t="inlineStr">
@@ -3808,7 +3808,7 @@
       </c>
       <c r="M16" s="8" t="inlineStr">
         <is>
-          <t>https://www.tsukasyuzou.jp/products/於多福-純米-1800ml</t>
+          <t>https://www.tsukasyuzou.jp/products/9代目於多福-すずかぜ-720ml</t>
         </is>
       </c>
     </row>

</xml_diff>